<commit_message>
fix: correct library URN typo (checklist_08-09--> checklist_09-08 & ref_id ( au ---> à la )
</commit_message>
<xml_diff>
--- a/tools/excel/dgssi/09-08/Checklist_Loi09-08.xlsx
+++ b/tools/excel/dgssi/09-08/Checklist_Loi09-08.xlsx
@@ -45,7 +45,7 @@
     <t xml:space="preserve">ref_id</t>
   </si>
   <si>
-    <t xml:space="preserve">Checklist des exigences relatives au loi 09-08</t>
+    <t xml:space="preserve">Checklist des exigences relatives à la loi 09-08</t>
   </si>
   <si>
     <t xml:space="preserve">name</t>
@@ -78,7 +78,7 @@
     <t xml:space="preserve">library</t>
   </si>
   <si>
-    <t xml:space="preserve">urn:bassou:risk:library:checklist_08-09</t>
+    <t xml:space="preserve">urn:bassou:risk:library:checklist_09-08</t>
   </si>
   <si>
     <t xml:space="preserve">version</t>

</xml_diff>

<commit_message>
fix: set parent section nodes to assessable: false (per @eric-intuitem feedback)
</commit_message>
<xml_diff>
--- a/tools/excel/dgssi/09-08/Checklist_Loi09-08.xlsx
+++ b/tools/excel/dgssi/09-08/Checklist_Loi09-08.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="req_meta" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="291">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -2094,9 +2094,7 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="A43" s="3"/>
       <c r="B43" s="3" t="n">
         <v>1</v>
       </c>
@@ -2482,9 +2480,7 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="A67" s="3"/>
       <c r="B67" s="3" t="n">
         <v>1</v>
       </c>
@@ -2877,9 +2873,7 @@
       </c>
     </row>
     <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="A92" s="3"/>
       <c r="B92" s="3" t="n">
         <v>2</v>
       </c>

</xml_diff>